<commit_message>
Update test data: Change login email to john@test.com
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata.xlsx
+++ b/src/test/resources/testdata.xlsx
@@ -441,7 +441,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>john5@test.com</t>
+          <t>john@test.com</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -488,7 +488,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>john5@test.com</t>
+          <t>john@test.com</t>
         </is>
       </c>
       <c r="C5" t="inlineStr"/>

</xml_diff>

<commit_message>
ci && step in testcase
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata.xlsx
+++ b/src/test/resources/testdata.xlsx
@@ -8,6 +8,9 @@
   </bookViews>
   <sheets>
     <sheet name="LoginData" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="RegisterData" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="UserProfileData" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="SearchData" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,13 +416,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:D5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>TestId</t>
+          <t>Key</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
@@ -430,6 +433,11 @@
       <c r="C1" t="inlineStr">
         <is>
           <t>Password</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Name</t>
         </is>
       </c>
     </row>
@@ -449,58 +457,307 @@
           <t>Abc12345</t>
         </is>
       </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>John Test</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>invalidEmail1</t>
+          <t>e2euser_09154559</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>test@</t>
+          <t>e2euser_09154559@test.com</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Abc12345</t>
+          <t>E2Epass!</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>E2E User</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>emptyEmail</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr"/>
+          <t>invalidEmail1</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>invalid-email</t>
+        </is>
+      </c>
       <c r="C4" t="inlineStr">
         <is>
           <t>Abc12345</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Invalid Email</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>emptyPassword</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
+          <t>emptyEmail</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr"/>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Abc12345</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Empty Email</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Email</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Password</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>John Test</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
         <is>
           <t>john@test.com</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr"/>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>bothEmpty</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr"/>
-      <c r="C6" t="inlineStr"/>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Abc12345</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>E2E User</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>e2euser_09154559@test.com</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>E2Epass!</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Generated User</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>generated@test.com</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>GenPass123</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Key</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Email</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Password</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Fullname</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Phone</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Address</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>valid_profile</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>john@test.com</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Abc12345</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>John Test</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>0912345678</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>123 Test Street, Hanoi</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>e2e_profile</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>e2euser_09154559@test.com</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>E2Epass!</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>E2E User</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>0900000000</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>456 Test Ave, HCMC</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Query</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>laptop</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>rtx 2050</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>headphones</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>